<commit_message>
Update test Excel export artifacts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/test_optimization_export.xlsx
+++ b/backend/test_optimization_export.xlsx
@@ -506,7 +506,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2025-12-15 07:23:25 UTC</t>
+          <t>Generated: 2026-02-24 12:43:05 UTC</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>d04abbea-2cf4-464e-90a9-437d87f411b9</t>
+          <t>db17d0fb-b114-48c9-9d8a-abb938ba8983</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
@@ -806,12 +806,12 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F2" s="8" t="n">
@@ -843,7 +843,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>0f482cec-764e-4ed8-9e36-115f7ce8a7f6</t>
+          <t>2b562fa4-ffc9-46a4-950b-676a622ff122</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F3" s="8" t="n">
@@ -895,7 +895,7 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>c15d5bc8-b441-4547-a411-fb56ce7286c4</t>
+          <t>08e176a8-3d59-4d7d-ac90-405fd6c0d4ac</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F4" s="8" t="n">
@@ -947,7 +947,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>1d86e3dd-aa37-4e50-999f-ba6c68f4615f</t>
+          <t>d724eb8d-9b80-4c19-b6b2-5b121f8fc6b6</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -962,12 +962,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F5" s="8" t="n">
@@ -999,7 +999,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>554f4b9c-0993-48b5-a472-4a825e95763b</t>
+          <t>370e0459-79d3-470d-b47f-eba860400e54</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -1014,12 +1014,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F6" s="8" t="n">
@@ -1051,7 +1051,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>a6ba832d-962d-44f0-a4e2-e6fe81945f26</t>
+          <t>b6902d63-4c54-41d1-863b-a8e3db976448</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F7" s="8" t="n">
@@ -1103,7 +1103,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>d7c4cc28-0dd7-44c7-a737-90441b44eece</t>
+          <t>27cdcfd0-3808-426d-ba66-a1de04e1adfc</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F8" s="8" t="n">
@@ -1155,7 +1155,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>eedd0b06-cb02-47ae-8c2b-224c4886888c</t>
+          <t>758a94ff-1124-491c-ba35-c589c005d744</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1170,12 +1170,12 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F9" s="8" t="n">
@@ -1207,7 +1207,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>a6a1e862-8b6c-49bd-8189-ed787a80e118</t>
+          <t>9ca802c9-d7e1-4c1b-9ed4-ccbf5d3b2c68</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1222,12 +1222,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F10" s="8" t="n">
@@ -1259,7 +1259,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>3dcae4e8-9290-4bb5-9858-1eaab0d49c34</t>
+          <t>1e01e4fa-aa58-43ee-8089-a6970776c248</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>2025-12-15 07:23:25</t>
+          <t>2026-02-24 12:43:05</t>
         </is>
       </c>
       <c r="F11" s="8" t="n">
@@ -2000,22 +2000,22 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
+          <t>sharpe_ratio</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>max_drawdown</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>total_return</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
           <t>volatility</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>sharpe_ratio</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>max_drawdown</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>total_return</t>
         </is>
       </c>
     </row>
@@ -2035,16 +2035,16 @@
         <v>0.1</v>
       </c>
       <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.15</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.05</v>
       </c>
     </row>
     <row r="4">
@@ -2063,16 +2063,16 @@
         <v>0.15</v>
       </c>
       <c r="E4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.09000000000000001</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.16</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.09000000000000001</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -2091,16 +2091,16 @@
         <v>0.2</v>
       </c>
       <c r="E5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H5" t="n">
         <v>0.17</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.09</v>
       </c>
     </row>
     <row r="6">
@@ -2119,16 +2119,16 @@
         <v>0.25</v>
       </c>
       <c r="E6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H6" t="n">
         <v>0.18</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.11</v>
       </c>
     </row>
     <row r="7">
@@ -2147,16 +2147,16 @@
         <v>0.3</v>
       </c>
       <c r="E7" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H7" t="n">
         <v>0.19</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.13</v>
       </c>
     </row>
     <row r="8">
@@ -2175,16 +2175,16 @@
         <v>0.35</v>
       </c>
       <c r="E8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.2</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.15</v>
       </c>
     </row>
     <row r="9">
@@ -2203,16 +2203,16 @@
         <v>0.4</v>
       </c>
       <c r="E9" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.04000000000000001</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H9" t="n">
         <v>0.21</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.04000000000000001</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.17</v>
       </c>
     </row>
     <row r="10">
@@ -2231,16 +2231,16 @@
         <v>0.4500000000000001</v>
       </c>
       <c r="E10" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.22</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.19</v>
       </c>
     </row>
     <row r="11">
@@ -2259,16 +2259,16 @@
         <v>0.5</v>
       </c>
       <c r="E11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H11" t="n">
         <v>0.23</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.21</v>
       </c>
     </row>
     <row r="12">
@@ -2287,16 +2287,16 @@
         <v>0.55</v>
       </c>
       <c r="E12" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.01000000000000001</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H12" t="n">
         <v>0.24</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.01000000000000001</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>